<commit_message>
chore(tracker): board refresh to-the-minute (post USERS/SC-CLUSTER/audit merges)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-03.xlsx
+++ b/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-03.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2875" uniqueCount="841">
   <si>
-    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-03 (verified vs origin/main + 1788 merged PRs)</t>
+    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-03 (verified vs origin/main + 1794 merged PRs)</t>
   </si>
   <si>
     <t>DONE = verified on main (branch merged or files present) · NEEDS-VERIFY = weak signal, not trusted until GUARD confirms · PENDING = needs build · PENDING (GATED) = financial/locked, needs Jorge's gate first</t>
@@ -12636,7 +12636,7 @@
         <v>839</v>
       </c>
       <c r="B9">
-        <v>1788</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -12644,7 +12644,7 @@
         <v>840</v>
       </c>
       <c r="B10">
-        <v>7688</v>
+        <v>7694</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(tracker): board refresh to-the-minute (post USERS/SC-CLUSTER/audit merges) (#1907)
Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-03.xlsx
+++ b/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-03.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2875" uniqueCount="841">
   <si>
-    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-03 (verified vs origin/main + 1788 merged PRs)</t>
+    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-03 (verified vs origin/main + 1794 merged PRs)</t>
   </si>
   <si>
     <t>DONE = verified on main (branch merged or files present) · NEEDS-VERIFY = weak signal, not trusted until GUARD confirms · PENDING = needs build · PENDING (GATED) = financial/locked, needs Jorge's gate first</t>
@@ -12636,7 +12636,7 @@
         <v>839</v>
       </c>
       <c r="B9">
-        <v>1788</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -12644,7 +12644,7 @@
         <v>840</v>
       </c>
       <c r="B10">
-        <v>7688</v>
+        <v>7694</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(program): refresh block-reconciliation snapshot 2026-07-03 (advance Program Board)
The Program Board (/api/v1/program/board) reads docs/trackers/block-reconciliation-data.json at
request time from the deployed code — so the board only advances when this committed snapshot is
refreshed + deployed. Re-ran reconcile:blocks: 476 blocks — DONE=436, NEEDS-VERIFY=3, PENDING=4,
PENDING(GATED)=33. Non-financial tracker data.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-03.xlsx
+++ b/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-03.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2875" uniqueCount="841">
   <si>
-    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-03 (verified vs origin/main + 1794 merged PRs)</t>
+    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-03 (verified vs origin/main + 1809 merged PRs)</t>
   </si>
   <si>
     <t>DONE = verified on main (branch merged or files present) · NEEDS-VERIFY = weak signal, not trusted until GUARD confirms · PENDING = needs build · PENDING (GATED) = financial/locked, needs Jorge's gate first</t>
@@ -12636,7 +12636,7 @@
         <v>839</v>
       </c>
       <c r="B9">
-        <v>1794</v>
+        <v>1809</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -12644,7 +12644,7 @@
         <v>840</v>
       </c>
       <c r="B10">
-        <v>7694</v>
+        <v>7703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(program): refresh block-reconciliation snapshot 2026-07-03 (advance Program Board) (#1921)
The Program Board (/api/v1/program/board) reads docs/trackers/block-reconciliation-data.json at
request time from the deployed code — so the board only advances when this committed snapshot is
refreshed + deployed. Re-ran reconcile:blocks: 476 blocks — DONE=436, NEEDS-VERIFY=3, PENDING=4,
PENDING(GATED)=33. Non-financial tracker data.

Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-03.xlsx
+++ b/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-03.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2875" uniqueCount="841">
   <si>
-    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-03 (verified vs origin/main + 1794 merged PRs)</t>
+    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-03 (verified vs origin/main + 1809 merged PRs)</t>
   </si>
   <si>
     <t>DONE = verified on main (branch merged or files present) · NEEDS-VERIFY = weak signal, not trusted until GUARD confirms · PENDING = needs build · PENDING (GATED) = financial/locked, needs Jorge's gate first</t>
@@ -12636,7 +12636,7 @@
         <v>839</v>
       </c>
       <c r="B9">
-        <v>1794</v>
+        <v>1809</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -12644,7 +12644,7 @@
         <v>840</v>
       </c>
       <c r="B10">
-        <v>7694</v>
+        <v>7703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(program): refresh block-reconciliation snapshot (PM) — merged-PR spine 1835
Re-ran reconcile:blocks after today's merges. Block counts unchanged (436 done / 40 open — the
banking/accounting/visual FIXES are PRs, not registered blocks, so Focus/Pending don't move);
merged-PR spine advanced 1813→1835 and the data-as-of stamp refreshes. Deploys so the Program
Board + Final Additions page read current data.
</commit_message>
<xml_diff>
--- a/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-03.xlsx
+++ b/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-03.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2875" uniqueCount="841">
   <si>
-    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-03 (verified vs origin/main + 1809 merged PRs)</t>
+    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-03 (verified vs origin/main + 1835 merged PRs)</t>
   </si>
   <si>
     <t>DONE = verified on main (branch merged or files present) · NEEDS-VERIFY = weak signal, not trusted until GUARD confirms · PENDING = needs build · PENDING (GATED) = financial/locked, needs Jorge's gate first</t>
@@ -12636,7 +12636,7 @@
         <v>839</v>
       </c>
       <c r="B9">
-        <v>1809</v>
+        <v>1835</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -12644,7 +12644,7 @@
         <v>840</v>
       </c>
       <c r="B10">
-        <v>7703</v>
+        <v>7709</v>
       </c>
     </row>
   </sheetData>

</xml_diff>